<commit_message>
corrected limits on angles for scattering plane accessibility calculations
</commit_message>
<xml_diff>
--- a/clino_hk0_plane_hkl.xlsx
+++ b/clino_hk0_plane_hkl.xlsx
@@ -500,7 +500,7 @@
       <c r="H2" t="n">
         <v>13</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" t="b">
         <v>0</v>
       </c>
     </row>
@@ -529,7 +529,7 @@
       <c r="H3" t="n">
         <v>13</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" t="b">
         <v>0</v>
       </c>
     </row>
@@ -558,7 +558,7 @@
       <c r="H4" t="n">
         <v>13</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" t="b">
         <v>0</v>
       </c>
     </row>
@@ -587,7 +587,7 @@
       <c r="H5" t="n">
         <v>13</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" t="b">
         <v>0</v>
       </c>
     </row>
@@ -616,7 +616,7 @@
       <c r="H6" t="n">
         <v>13</v>
       </c>
-      <c r="I6" t="n">
+      <c r="I6" t="b">
         <v>0</v>
       </c>
     </row>
@@ -645,7 +645,7 @@
       <c r="H7" t="n">
         <v>13</v>
       </c>
-      <c r="I7" t="n">
+      <c r="I7" t="b">
         <v>0</v>
       </c>
     </row>
@@ -674,7 +674,7 @@
       <c r="H8" t="n">
         <v>13</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" t="b">
         <v>0</v>
       </c>
     </row>
@@ -703,7 +703,7 @@
       <c r="H9" t="n">
         <v>13</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" t="b">
         <v>0</v>
       </c>
     </row>
@@ -732,7 +732,7 @@
       <c r="H10" t="n">
         <v>13</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" t="b">
         <v>0</v>
       </c>
     </row>
@@ -761,7 +761,7 @@
       <c r="H11" t="n">
         <v>13</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" t="b">
         <v>0</v>
       </c>
     </row>
@@ -790,7 +790,7 @@
       <c r="H12" t="n">
         <v>13</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -819,7 +819,7 @@
       <c r="H13" t="n">
         <v>13</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" t="b">
         <v>0</v>
       </c>
     </row>
@@ -848,7 +848,7 @@
       <c r="H14" t="n">
         <v>13</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -877,7 +877,7 @@
       <c r="H15" t="n">
         <v>13</v>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" t="b">
         <v>0</v>
       </c>
     </row>
@@ -906,7 +906,7 @@
       <c r="H16" t="n">
         <v>13</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" t="b">
         <v>0</v>
       </c>
     </row>
@@ -935,7 +935,7 @@
       <c r="H17" t="n">
         <v>13</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -964,7 +964,7 @@
       <c r="H18" t="n">
         <v>13</v>
       </c>
-      <c r="I18" t="n">
+      <c r="I18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -993,7 +993,7 @@
       <c r="H19" t="n">
         <v>13</v>
       </c>
-      <c r="I19" t="n">
+      <c r="I19" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       <c r="H20" t="n">
         <v>13</v>
       </c>
-      <c r="I20" t="n">
+      <c r="I20" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       <c r="H21" t="n">
         <v>13</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I21" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       <c r="H22" t="n">
         <v>13</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I22" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       <c r="H23" t="n">
         <v>13</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I23" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       <c r="H24" t="n">
         <v>13</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I24" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       <c r="H25" t="n">
         <v>13</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I25" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       <c r="H26" t="n">
         <v>13</v>
       </c>
-      <c r="I26" t="n">
+      <c r="I26" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       <c r="H27" t="n">
         <v>13</v>
       </c>
-      <c r="I27" t="n">
+      <c r="I27" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       <c r="H28" t="n">
         <v>13</v>
       </c>
-      <c r="I28" t="n">
+      <c r="I28" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
       <c r="H29" t="n">
         <v>13</v>
       </c>
-      <c r="I29" t="n">
+      <c r="I29" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       <c r="H30" t="n">
         <v>13</v>
       </c>
-      <c r="I30" t="n">
+      <c r="I30" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       <c r="H31" t="n">
         <v>13</v>
       </c>
-      <c r="I31" t="n">
+      <c r="I31" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       <c r="H32" t="n">
         <v>13</v>
       </c>
-      <c r="I32" t="n">
+      <c r="I32" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1399,7 +1399,7 @@
       <c r="H33" t="n">
         <v>13</v>
       </c>
-      <c r="I33" t="n">
+      <c r="I33" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       <c r="H34" t="n">
         <v>13</v>
       </c>
-      <c r="I34" t="n">
+      <c r="I34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
       <c r="H35" t="n">
         <v>13</v>
       </c>
-      <c r="I35" t="n">
+      <c r="I35" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1486,7 +1486,7 @@
       <c r="H36" t="n">
         <v>13</v>
       </c>
-      <c r="I36" t="n">
+      <c r="I36" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
       <c r="H37" t="n">
         <v>13</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I37" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       <c r="H38" t="n">
         <v>13</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I38" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       <c r="H39" t="n">
         <v>13</v>
       </c>
-      <c r="I39" t="n">
+      <c r="I39" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1602,7 +1602,7 @@
       <c r="H40" t="n">
         <v>13</v>
       </c>
-      <c r="I40" t="n">
+      <c r="I40" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       <c r="H41" t="n">
         <v>13</v>
       </c>
-      <c r="I41" t="n">
+      <c r="I41" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       <c r="H42" t="n">
         <v>13</v>
       </c>
-      <c r="I42" t="n">
+      <c r="I42" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       <c r="H43" t="n">
         <v>13</v>
       </c>
-      <c r="I43" t="n">
+      <c r="I43" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       <c r="H44" t="n">
         <v>13</v>
       </c>
-      <c r="I44" t="n">
+      <c r="I44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1747,7 +1747,7 @@
       <c r="H45" t="n">
         <v>13</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I45" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       <c r="H46" t="n">
         <v>13</v>
       </c>
-      <c r="I46" t="n">
+      <c r="I46" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1805,7 +1805,7 @@
       <c r="H47" t="n">
         <v>13</v>
       </c>
-      <c r="I47" t="n">
+      <c r="I47" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       <c r="H48" t="n">
         <v>13</v>
       </c>
-      <c r="I48" t="n">
+      <c r="I48" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       <c r="H49" t="n">
         <v>13</v>
       </c>
-      <c r="I49" t="n">
+      <c r="I49" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       <c r="H50" t="n">
         <v>13</v>
       </c>
-      <c r="I50" t="n">
+      <c r="I50" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>